<commit_message>
Export known product stock and exact clickable variant image links
</commit_message>
<xml_diff>
--- a/ChotuApp_Template.xlsx
+++ b/ChotuApp_Template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brand Info" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Products" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Product Images" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Option Groups" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Options" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Enrichment Notes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Variant Combinations" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Variant Mapping Guide" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Info" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Images" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Option Groups" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enrichment Notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variant Combinations" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variant Mapping Guide" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1071,6 +1071,7 @@
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1162,6 +1163,11 @@
       <c r="R1" s="6" t="inlineStr">
         <is>
           <t>source_url</t>
+        </is>
+      </c>
+      <c r="S1" s="6" t="inlineStr">
+        <is>
+          <t>stock_quantity (kitni quantity bechni hai)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add optional store category and product ranking fields to import templates
</commit_message>
<xml_diff>
--- a/ChotuApp_Template.xlsx
+++ b/ChotuApp_Template.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enrichment Notes" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variant Combinations" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variant Mapping Guide" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranking Guide" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -97,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +141,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -223,6 +227,41 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ChotuApp</author>
+  </authors>
+  <commentList>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional positive integer; lower numbers appear first. Store-specific category merchandising priority, not a sales claim. Use the same value for every product in that category within a shop. Blank means unassigned.</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional positive integer; lower numbers appear first within the category. Set only from documented evidence or explicit manual selection. Blank means unranked.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional: store_bestseller, external_trend, or manual_selection. External popularity is not proof of this shop’s sales. Blank means no ranking evidence recorded.</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Evidence page URL. Required for store_bestseller and external_trend; do not substitute the product URL unless it actually documents the ranking.</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>Date/time when the evidence was actually checked, preferably ISO 8601 with timezone. Leave blank until checked; do not invent freshness.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -443,12 +482,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B41"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -463,6 +503,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -484,6 +525,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -519,6 +561,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -547,6 +590,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -568,6 +612,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -582,6 +627,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -596,6 +642,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -624,6 +671,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -631,6 +679,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="3" t="inlineStr">
         <is>
@@ -668,6 +717,160 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="n"/>
+      <c r="B1" s="25" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Field / Topic</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>Importer and storefront contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>category_priority</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>Optional positive integer; lower numbers appear first. Store-specific category merchandising priority, not a sales claim. Use the same value for every product in that category within a shop. Blank means unassigned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>product_priority</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Optional positive integer; lower numbers appear first within the category. Set only from documented evidence or explicit manual selection. Blank means unranked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>popularity_basis</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Optional: store_bestseller, external_trend, or manual_selection. External popularity is not proof of this shop’s sales. Blank means no ranking evidence recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>popularity_source_url</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Evidence page URL. Required for store_bestseller and external_trend; do not substitute the product URL unless it actually documents the ranking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>popularity_checked_at</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>Date/time when the evidence was actually checked, preferably ISO 8601 with timezone. Leave blank until checked; do not invent freshness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Default display order</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Within the shop: category_priority ascending, with blank priorities last; ties preserve existing category order. Within each category: product_priority ascending, blanks last; then valid payable product price ascending; equal prices: genuine discount descending, then original import order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>Evidence validation</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Reject unsupported basis values. Require an actual evidence URL and checked timestamp for store_bestseller/external_trend. Do not generate a best-selling badge from external_trend or manual_selection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Category consistency</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Validate one consistent category_priority per shop/category. Do not let alphabetical category ordering put unrelated side categories ahead of the shop’s primary categories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Compatibility</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>All ranking fields are optional. Preserve blank values as null. Existing product, stock, price, shop_code, variants and image columns retain their existing meaning. Column matching must use header names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>These columns store ranking evidence and priorities. Template updates alone do not collect bestseller evidence, change an active cloud worker, or update the website importer/storefront.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1051,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1072,6 +1275,11 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="34" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="22" max="22"/>
+    <col width="55" customWidth="1" min="23" max="23"/>
+    <col width="25" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1168,6 +1376,31 @@
       <c r="S1" s="6" t="inlineStr">
         <is>
           <t>stock_quantity (kitni quantity bechni hai)</t>
+        </is>
+      </c>
+      <c r="T1" s="6" t="inlineStr">
+        <is>
+          <t>category_priority</t>
+        </is>
+      </c>
+      <c r="U1" s="6" t="inlineStr">
+        <is>
+          <t>product_priority</t>
+        </is>
+      </c>
+      <c r="V1" s="6" t="inlineStr">
+        <is>
+          <t>popularity_basis</t>
+        </is>
+      </c>
+      <c r="W1" s="6" t="inlineStr">
+        <is>
+          <t>popularity_source_url</t>
+        </is>
+      </c>
+      <c r="X1" s="6" t="inlineStr">
+        <is>
+          <t>popularity_checked_at</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1410,7 @@
       <formula>AND($A2&lt;&gt;"",COUNTIF($A$2:$A$5000,$A2)&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="7">
     <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Galat value" error="Sirf new ya used likhein" type="list">
       <formula1>"new,used"</formula1>
     </dataValidation>
@@ -1190,8 +1423,18 @@
     <dataValidation sqref="J2:J5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Galat value" error="Warranty mahine ka number ho" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
+    <dataValidation sqref="T2:T1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid priority" error="Use a positive whole number or leave blank." type="whole" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid priority" error="Use a positive whole number or leave blank." type="whole" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V1048576" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"store_bestseller,external_trend,manual_selection"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add per-product analysis notes with scoped website labels and collection evidence
</commit_message>
<xml_diff>
--- a/ChotuApp_Template.xlsx
+++ b/ChotuApp_Template.xlsx
@@ -260,6 +260,11 @@
         <t>Date/time when the evidence was actually checked, preferably ISO 8601 with timezone. Leave blank until checked; do not invent freshness.</t>
       </text>
     </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>Internal Rule 804 research note: record observed bestseller-sort position, product-page merchant labels, named collection membership, source URLs, check times and uncertainty. Top/featured collection names alone do not prove sales. Preserve as plain text; do not display automatically as customer product description.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -726,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -866,6 +871,18 @@
       <c r="B12" s="25" t="inlineStr">
         <is>
           <t>These columns store ranking evidence and priorities. Template updates alone do not collect bestseller evidence, change an active cloud worker, or update the website importer/storefront.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>analysis_note</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Internal Rule 804 research note: record observed bestseller-sort position, product-page merchant labels, named collection membership, source URLs, check times and uncertainty. Top/featured collection names alone do not prove sales. Preserve as plain text; do not display automatically as customer product description.</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1280,6 +1297,7 @@
     <col width="25" customWidth="1" min="22" max="22"/>
     <col width="55" customWidth="1" min="23" max="23"/>
     <col width="25" customWidth="1" min="24" max="24"/>
+    <col width="80" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1401,6 +1419,11 @@
       <c r="X1" s="6" t="inlineStr">
         <is>
           <t>popularity_checked_at</t>
+        </is>
+      </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t>analysis_note</t>
         </is>
       </c>
     </row>

</xml_diff>